<commit_message>
added zom feature to graph and scoring
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1163,6 +1163,120 @@
       <c r="J19" t="inlineStr">
         <is>
           <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>693.6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>696.51</v>
+      </c>
+      <c r="E20" t="n">
+        <v>685.76</v>
+      </c>
+      <c r="F20" t="n">
+        <v>692.96</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="H20" t="n">
+        <v>684.54</v>
+      </c>
+      <c r="I20" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>690.83</v>
+      </c>
+      <c r="D21" t="n">
+        <v>690.83</v>
+      </c>
+      <c r="E21" t="n">
+        <v>683.48</v>
+      </c>
+      <c r="F21" t="n">
+        <v>683.48</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="H21" t="n">
+        <v>684.54</v>
+      </c>
+      <c r="I21" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:24</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>688.0700000000001</v>
+      </c>
+      <c r="D22" t="n">
+        <v>688.0700000000001</v>
+      </c>
+      <c r="E22" t="n">
+        <v>674.91</v>
+      </c>
+      <c r="F22" t="n">
+        <v>674.91</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-1.41</v>
+      </c>
+      <c r="H22" t="n">
+        <v>684.54</v>
+      </c>
+      <c r="I22" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1913,6 +2027,120 @@
       <c r="J19" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>266.12</v>
+      </c>
+      <c r="D20" t="n">
+        <v>277.25</v>
+      </c>
+      <c r="E20" t="n">
+        <v>260.01</v>
+      </c>
+      <c r="F20" t="n">
+        <v>273.19</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="H20" t="n">
+        <v>268.09</v>
+      </c>
+      <c r="I20" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>264.27</v>
+      </c>
+      <c r="D21" t="n">
+        <v>270.08</v>
+      </c>
+      <c r="E21" t="n">
+        <v>260.01</v>
+      </c>
+      <c r="F21" t="n">
+        <v>266.13</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="H21" t="n">
+        <v>268.09</v>
+      </c>
+      <c r="I21" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>262.42</v>
+      </c>
+      <c r="D22" t="n">
+        <v>270.08</v>
+      </c>
+      <c r="E22" t="n">
+        <v>254.91</v>
+      </c>
+      <c r="F22" t="n">
+        <v>260.91</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-2.68</v>
+      </c>
+      <c r="H22" t="n">
+        <v>268.09</v>
+      </c>
+      <c r="I22" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
     </row>
@@ -1927,7 +2155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2666,6 +2894,120 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>419.86</v>
+      </c>
+      <c r="D20" t="n">
+        <v>421.96</v>
+      </c>
+      <c r="E20" t="n">
+        <v>396.18</v>
+      </c>
+      <c r="F20" t="n">
+        <v>396.18</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H20" t="n">
+        <v>395.04</v>
+      </c>
+      <c r="I20" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>415.64</v>
+      </c>
+      <c r="D21" t="n">
+        <v>415.64</v>
+      </c>
+      <c r="E21" t="n">
+        <v>382.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>382.7</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="H21" t="n">
+        <v>395.04</v>
+      </c>
+      <c r="I21" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-02-28 01:38:25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>411.41</v>
+      </c>
+      <c r="D22" t="n">
+        <v>411.41</v>
+      </c>
+      <c r="E22" t="n">
+        <v>370.51</v>
+      </c>
+      <c r="F22" t="n">
+        <v>370.51</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-6.21</v>
+      </c>
+      <c r="H22" t="n">
+        <v>395.04</v>
+      </c>
+      <c r="I22" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
bug fixes, and changed format of model storage
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,36 @@
           <t>Signal</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Error %</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dir Accuracy %</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>In Range %</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Matched Preds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1277,6 +1307,348 @@
       <c r="J22" t="inlineStr">
         <is>
           <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>678.16</v>
+      </c>
+      <c r="D23" t="n">
+        <v>694.96</v>
+      </c>
+      <c r="E23" t="n">
+        <v>668.79</v>
+      </c>
+      <c r="F23" t="n">
+        <v>691.83</v>
+      </c>
+      <c r="G23" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="H23" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I23" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>674.5700000000001</v>
+      </c>
+      <c r="D24" t="n">
+        <v>683.54</v>
+      </c>
+      <c r="E24" t="n">
+        <v>668.79</v>
+      </c>
+      <c r="F24" t="n">
+        <v>680.45</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="H24" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I24" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>670.97</v>
+      </c>
+      <c r="D25" t="n">
+        <v>683.54</v>
+      </c>
+      <c r="E25" t="n">
+        <v>656.4299999999999</v>
+      </c>
+      <c r="F25" t="n">
+        <v>667.88</v>
+      </c>
+      <c r="G25" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H25" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I25" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>665.04</v>
+      </c>
+      <c r="D26" t="n">
+        <v>706.11</v>
+      </c>
+      <c r="E26" t="n">
+        <v>665.04</v>
+      </c>
+      <c r="F26" t="n">
+        <v>681.6</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="H26" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I26" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>661.51</v>
+      </c>
+      <c r="D27" t="n">
+        <v>694.5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>661.51</v>
+      </c>
+      <c r="F27" t="n">
+        <v>670.39</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="H27" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I27" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>657.98</v>
+      </c>
+      <c r="D28" t="n">
+        <v>694.5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>657.98</v>
+      </c>
+      <c r="F28" t="n">
+        <v>658</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I28" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>687.9400000000001</v>
+      </c>
+      <c r="D29" t="n">
+        <v>694.4299999999999</v>
+      </c>
+      <c r="E29" t="n">
+        <v>662.15</v>
+      </c>
+      <c r="F29" t="n">
+        <v>662.15</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="H29" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I29" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>684.29</v>
+      </c>
+      <c r="D30" t="n">
+        <v>690.02</v>
+      </c>
+      <c r="E30" t="n">
+        <v>651.26</v>
+      </c>
+      <c r="F30" t="n">
+        <v>651.26</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H30" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I30" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>680.64</v>
+      </c>
+      <c r="D31" t="n">
+        <v>683.01</v>
+      </c>
+      <c r="E31" t="n">
+        <v>639.22</v>
+      </c>
+      <c r="F31" t="n">
+        <v>639.22</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="H31" t="n">
+        <v>645.09</v>
+      </c>
+      <c r="I31" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1345,6 +1717,36 @@
           <t>Signal</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Error %</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dir Accuracy %</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>In Range %</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Matched Preds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2141,6 +2543,348 @@
       <c r="J22" t="inlineStr">
         <is>
           <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>273.85</v>
+      </c>
+      <c r="D23" t="n">
+        <v>275.33</v>
+      </c>
+      <c r="E23" t="n">
+        <v>264.21</v>
+      </c>
+      <c r="F23" t="n">
+        <v>275.33</v>
+      </c>
+      <c r="G23" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="H23" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I23" t="n">
+        <v>80</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>272.55</v>
+      </c>
+      <c r="D24" t="n">
+        <v>272.55</v>
+      </c>
+      <c r="E24" t="n">
+        <v>264.21</v>
+      </c>
+      <c r="F24" t="n">
+        <v>270.87</v>
+      </c>
+      <c r="G24" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="H24" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I24" t="n">
+        <v>80</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>271.26</v>
+      </c>
+      <c r="D25" t="n">
+        <v>271.26</v>
+      </c>
+      <c r="E25" t="n">
+        <v>260.28</v>
+      </c>
+      <c r="F25" t="n">
+        <v>266.83</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="H25" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I25" t="n">
+        <v>80</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>257.1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>273.75</v>
+      </c>
+      <c r="E26" t="n">
+        <v>256</v>
+      </c>
+      <c r="F26" t="n">
+        <v>263.77</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I26" t="n">
+        <v>80</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>255.88</v>
+      </c>
+      <c r="D27" t="n">
+        <v>269.32</v>
+      </c>
+      <c r="E27" t="n">
+        <v>255.88</v>
+      </c>
+      <c r="F27" t="n">
+        <v>259.5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="H27" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I27" t="n">
+        <v>80</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>254.66</v>
+      </c>
+      <c r="D28" t="n">
+        <v>269.32</v>
+      </c>
+      <c r="E28" t="n">
+        <v>252.18</v>
+      </c>
+      <c r="F28" t="n">
+        <v>255.63</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="H28" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I28" t="n">
+        <v>80</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>266.08</v>
+      </c>
+      <c r="D29" t="n">
+        <v>266.08</v>
+      </c>
+      <c r="E29" t="n">
+        <v>261.18</v>
+      </c>
+      <c r="F29" t="n">
+        <v>261.73</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H29" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I29" t="n">
+        <v>80</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>264.82</v>
+      </c>
+      <c r="D30" t="n">
+        <v>264.82</v>
+      </c>
+      <c r="E30" t="n">
+        <v>257.49</v>
+      </c>
+      <c r="F30" t="n">
+        <v>257.49</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="H30" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I30" t="n">
+        <v>80</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>263.56</v>
+      </c>
+      <c r="D31" t="n">
+        <v>263.56</v>
+      </c>
+      <c r="E31" t="n">
+        <v>253.65</v>
+      </c>
+      <c r="F31" t="n">
+        <v>253.65</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H31" t="n">
+        <v>252.89</v>
+      </c>
+      <c r="I31" t="n">
+        <v>80</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2209,6 +2953,36 @@
           <t>Signal</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Error %</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Dir Accuracy %</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>In Range %</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Matched Preds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2247,6 +3021,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2285,6 +3065,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2323,6 +3109,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2361,6 +3153,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2399,6 +3197,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2437,6 +3241,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2475,6 +3285,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2513,6 +3329,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2551,6 +3373,12 @@
           <t>STRONG BUY</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2589,6 +3417,12 @@
           <t>BUY</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2627,6 +3461,12 @@
           <t>BUY</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2665,6 +3505,12 @@
           <t>BUY</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2703,6 +3549,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2741,6 +3593,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2779,6 +3637,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2817,6 +3681,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2855,6 +3725,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2893,6 +3769,12 @@
           <t>HOLD</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2931,6 +3813,12 @@
           <t>SELL</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2969,6 +3857,12 @@
           <t>SELL</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3007,6 +3901,408 @@
           <t>SELL</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>388.46</v>
+      </c>
+      <c r="D23" t="n">
+        <v>455.39</v>
+      </c>
+      <c r="E23" t="n">
+        <v>388.46</v>
+      </c>
+      <c r="F23" t="n">
+        <v>455.39</v>
+      </c>
+      <c r="G23" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="H23" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I23" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>386.23</v>
+      </c>
+      <c r="D24" t="n">
+        <v>446.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>386.23</v>
+      </c>
+      <c r="F24" t="n">
+        <v>446.48</v>
+      </c>
+      <c r="G24" t="n">
+        <v>22</v>
+      </c>
+      <c r="H24" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I24" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:41:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>384.01</v>
+      </c>
+      <c r="D25" t="n">
+        <v>438.41</v>
+      </c>
+      <c r="E25" t="n">
+        <v>384.01</v>
+      </c>
+      <c r="F25" t="n">
+        <v>438.41</v>
+      </c>
+      <c r="G25" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="H25" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I25" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>365.54</v>
+      </c>
+      <c r="D26" t="n">
+        <v>382.93</v>
+      </c>
+      <c r="E26" t="n">
+        <v>365.54</v>
+      </c>
+      <c r="F26" t="n">
+        <v>382.93</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="H26" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I26" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>363.44</v>
+      </c>
+      <c r="D27" t="n">
+        <v>375.44</v>
+      </c>
+      <c r="E27" t="n">
+        <v>363.44</v>
+      </c>
+      <c r="F27" t="n">
+        <v>375.44</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="H27" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I27" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:46:20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>361.35</v>
+      </c>
+      <c r="D28" t="n">
+        <v>374.61</v>
+      </c>
+      <c r="E28" t="n">
+        <v>361.35</v>
+      </c>
+      <c r="F28" t="n">
+        <v>368.66</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="H28" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I28" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>401.16</v>
+      </c>
+      <c r="D29" t="n">
+        <v>414.18</v>
+      </c>
+      <c r="E29" t="n">
+        <v>396.7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>396.7</v>
+      </c>
+      <c r="G29" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H29" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I29" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>398.86</v>
+      </c>
+      <c r="D30" t="n">
+        <v>410.69</v>
+      </c>
+      <c r="E30" t="n">
+        <v>388.94</v>
+      </c>
+      <c r="F30" t="n">
+        <v>388.94</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="H30" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I30" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>396.56</v>
+      </c>
+      <c r="D31" t="n">
+        <v>406.08</v>
+      </c>
+      <c r="E31" t="n">
+        <v>381.92</v>
+      </c>
+      <c r="F31" t="n">
+        <v>381.92</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="H31" t="n">
+        <v>365.97</v>
+      </c>
+      <c r="I31" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
did a clean of the models and fixed the ui
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2106,6 +2106,234 @@
       <c r="J43" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>634.96</v>
+      </c>
+      <c r="D44" t="n">
+        <v>673.78</v>
+      </c>
+      <c r="E44" t="n">
+        <v>634.96</v>
+      </c>
+      <c r="F44" t="n">
+        <v>673.78</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H44" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I44" t="n">
+        <v>80</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>630.02</v>
+      </c>
+      <c r="D45" t="n">
+        <v>656.01</v>
+      </c>
+      <c r="E45" t="n">
+        <v>630.02</v>
+      </c>
+      <c r="F45" t="n">
+        <v>654.3200000000001</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="H45" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I45" t="n">
+        <v>80</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>625.09</v>
+      </c>
+      <c r="D46" t="n">
+        <v>649.47</v>
+      </c>
+      <c r="E46" t="n">
+        <v>625.09</v>
+      </c>
+      <c r="F46" t="n">
+        <v>639.9299999999999</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="H46" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I46" t="n">
+        <v>80</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>633.22</v>
+      </c>
+      <c r="D47" t="n">
+        <v>669.78</v>
+      </c>
+      <c r="E47" t="n">
+        <v>633.22</v>
+      </c>
+      <c r="F47" t="n">
+        <v>669.78</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="H47" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I47" t="n">
+        <v>80</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>628.29</v>
+      </c>
+      <c r="D48" t="n">
+        <v>654.86</v>
+      </c>
+      <c r="E48" t="n">
+        <v>628.29</v>
+      </c>
+      <c r="F48" t="n">
+        <v>650.4299999999999</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="H48" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I48" t="n">
+        <v>80</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>623.37</v>
+      </c>
+      <c r="D49" t="n">
+        <v>645.64</v>
+      </c>
+      <c r="E49" t="n">
+        <v>623.37</v>
+      </c>
+      <c r="F49" t="n">
+        <v>636.13</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="H49" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I49" t="n">
+        <v>80</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3798,6 +4026,234 @@
       <c r="J43" t="inlineStr">
         <is>
           <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>249.97</v>
+      </c>
+      <c r="D44" t="n">
+        <v>258.91</v>
+      </c>
+      <c r="E44" t="n">
+        <v>231.73</v>
+      </c>
+      <c r="F44" t="n">
+        <v>247.25</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-4.49</v>
+      </c>
+      <c r="H44" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I44" t="n">
+        <v>80</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>248.13</v>
+      </c>
+      <c r="D45" t="n">
+        <v>251.82</v>
+      </c>
+      <c r="E45" t="n">
+        <v>231.73</v>
+      </c>
+      <c r="F45" t="n">
+        <v>240.48</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-7.1</v>
+      </c>
+      <c r="H45" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I45" t="n">
+        <v>80</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>246.29</v>
+      </c>
+      <c r="D46" t="n">
+        <v>251.82</v>
+      </c>
+      <c r="E46" t="n">
+        <v>226.9</v>
+      </c>
+      <c r="F46" t="n">
+        <v>235.47</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-9.039999999999999</v>
+      </c>
+      <c r="H46" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I46" t="n">
+        <v>80</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>249.74</v>
+      </c>
+      <c r="D47" t="n">
+        <v>256.37</v>
+      </c>
+      <c r="E47" t="n">
+        <v>232.17</v>
+      </c>
+      <c r="F47" t="n">
+        <v>246.03</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-4.96</v>
+      </c>
+      <c r="H47" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I47" t="n">
+        <v>80</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>247.9</v>
+      </c>
+      <c r="D48" t="n">
+        <v>249.35</v>
+      </c>
+      <c r="E48" t="n">
+        <v>232.17</v>
+      </c>
+      <c r="F48" t="n">
+        <v>239.29</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-7.56</v>
+      </c>
+      <c r="H48" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I48" t="n">
+        <v>80</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>246.06</v>
+      </c>
+      <c r="D49" t="n">
+        <v>249.35</v>
+      </c>
+      <c r="E49" t="n">
+        <v>227.34</v>
+      </c>
+      <c r="F49" t="n">
+        <v>234.31</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-9.48</v>
+      </c>
+      <c r="H49" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I49" t="n">
+        <v>80</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -3812,7 +4268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5490,6 +5946,234 @@
       <c r="J43" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>351.61</v>
+      </c>
+      <c r="D44" t="n">
+        <v>381.18</v>
+      </c>
+      <c r="E44" t="n">
+        <v>324.97</v>
+      </c>
+      <c r="F44" t="n">
+        <v>324.97</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-12.85</v>
+      </c>
+      <c r="H44" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I44" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>348.44</v>
+      </c>
+      <c r="D45" t="n">
+        <v>368.47</v>
+      </c>
+      <c r="E45" t="n">
+        <v>314.13</v>
+      </c>
+      <c r="F45" t="n">
+        <v>314.13</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-15.75</v>
+      </c>
+      <c r="H45" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I45" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>345.27</v>
+      </c>
+      <c r="D46" t="n">
+        <v>368.47</v>
+      </c>
+      <c r="E46" t="n">
+        <v>306.12</v>
+      </c>
+      <c r="F46" t="n">
+        <v>306.12</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-17.9</v>
+      </c>
+      <c r="H46" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I46" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>374.42</v>
+      </c>
+      <c r="D47" t="n">
+        <v>438.78</v>
+      </c>
+      <c r="E47" t="n">
+        <v>370.38</v>
+      </c>
+      <c r="F47" t="n">
+        <v>370.38</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="H47" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I47" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>371.04</v>
+      </c>
+      <c r="D48" t="n">
+        <v>424.14</v>
+      </c>
+      <c r="E48" t="n">
+        <v>358.02</v>
+      </c>
+      <c r="F48" t="n">
+        <v>358.02</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-3.98</v>
+      </c>
+      <c r="H48" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I48" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>367.67</v>
+      </c>
+      <c r="D49" t="n">
+        <v>424.14</v>
+      </c>
+      <c r="E49" t="n">
+        <v>348.89</v>
+      </c>
+      <c r="F49" t="n">
+        <v>348.89</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="H49" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I49" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
     </row>
@@ -5504,7 +6188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5985,6 +6669,270 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>211.26</v>
+      </c>
+      <c r="D11" t="n">
+        <v>223.13</v>
+      </c>
+      <c r="E11" t="n">
+        <v>202.76</v>
+      </c>
+      <c r="F11" t="n">
+        <v>222.37</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I11" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>208.62</v>
+      </c>
+      <c r="D12" t="n">
+        <v>212.91</v>
+      </c>
+      <c r="E12" t="n">
+        <v>202.76</v>
+      </c>
+      <c r="F12" t="n">
+        <v>212.19</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="H12" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I12" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:40:24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>205.98</v>
+      </c>
+      <c r="D13" t="n">
+        <v>212.91</v>
+      </c>
+      <c r="E13" t="n">
+        <v>195.57</v>
+      </c>
+      <c r="F13" t="n">
+        <v>204.66</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="H13" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I13" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>234.26</v>
+      </c>
+      <c r="D14" t="n">
+        <v>240.82</v>
+      </c>
+      <c r="E14" t="n">
+        <v>224.97</v>
+      </c>
+      <c r="F14" t="n">
+        <v>238.37</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="H14" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I14" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>231.33</v>
+      </c>
+      <c r="D15" t="n">
+        <v>231.33</v>
+      </c>
+      <c r="E15" t="n">
+        <v>224.97</v>
+      </c>
+      <c r="F15" t="n">
+        <v>227.45</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="H15" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I15" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-07 17:44:19</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>228.4</v>
+      </c>
+      <c r="D16" t="n">
+        <v>229.79</v>
+      </c>
+      <c r="E16" t="n">
+        <v>216.99</v>
+      </c>
+      <c r="F16" t="n">
+        <v>219.38</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I16" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactored the project to be more modular for testing and debugging
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2332,6 +2332,120 @@
         <v>80</v>
       </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>633.73</v>
+      </c>
+      <c r="D50" t="n">
+        <v>668.26</v>
+      </c>
+      <c r="E50" t="n">
+        <v>633.73</v>
+      </c>
+      <c r="F50" t="n">
+        <v>668.26</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="H50" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I50" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>628.8</v>
+      </c>
+      <c r="D51" t="n">
+        <v>654.3200000000001</v>
+      </c>
+      <c r="E51" t="n">
+        <v>628.8</v>
+      </c>
+      <c r="F51" t="n">
+        <v>648.95</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-1.51</v>
+      </c>
+      <c r="H51" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I51" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>623.87</v>
+      </c>
+      <c r="D52" t="n">
+        <v>644.3200000000001</v>
+      </c>
+      <c r="E52" t="n">
+        <v>623.87</v>
+      </c>
+      <c r="F52" t="n">
+        <v>634.6799999999999</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-3.68</v>
+      </c>
+      <c r="H52" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I52" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -2348,7 +2462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4254,6 +4368,120 @@
       <c r="J49" t="inlineStr">
         <is>
           <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>257.01</v>
+      </c>
+      <c r="D50" t="n">
+        <v>275.13</v>
+      </c>
+      <c r="E50" t="n">
+        <v>240.71</v>
+      </c>
+      <c r="F50" t="n">
+        <v>268.01</v>
+      </c>
+      <c r="G50" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H50" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I50" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>255.11</v>
+      </c>
+      <c r="D51" t="n">
+        <v>267.6</v>
+      </c>
+      <c r="E51" t="n">
+        <v>240.71</v>
+      </c>
+      <c r="F51" t="n">
+        <v>260.67</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H51" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I51" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>253.22</v>
+      </c>
+      <c r="D52" t="n">
+        <v>267.6</v>
+      </c>
+      <c r="E52" t="n">
+        <v>235.7</v>
+      </c>
+      <c r="F52" t="n">
+        <v>255.24</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="H52" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I52" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6174,6 +6402,120 @@
       <c r="J49" t="inlineStr">
         <is>
           <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>353.78</v>
+      </c>
+      <c r="D50" t="n">
+        <v>428.04</v>
+      </c>
+      <c r="E50" t="n">
+        <v>353.78</v>
+      </c>
+      <c r="F50" t="n">
+        <v>355</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="H50" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I50" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>350.59</v>
+      </c>
+      <c r="D51" t="n">
+        <v>413.76</v>
+      </c>
+      <c r="E51" t="n">
+        <v>343.15</v>
+      </c>
+      <c r="F51" t="n">
+        <v>343.15</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-7.97</v>
+      </c>
+      <c r="H51" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I51" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>347.4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>413.76</v>
+      </c>
+      <c r="E52" t="n">
+        <v>334.4</v>
+      </c>
+      <c r="F52" t="n">
+        <v>334.4</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-10.32</v>
+      </c>
+      <c r="H52" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I52" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6933,6 +7275,138 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>227.13</v>
+      </c>
+      <c r="D17" t="n">
+        <v>245.28</v>
+      </c>
+      <c r="E17" t="n">
+        <v>210.45</v>
+      </c>
+      <c r="F17" t="n">
+        <v>245.28</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="H17" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I17" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>224.29</v>
+      </c>
+      <c r="D18" t="n">
+        <v>234.05</v>
+      </c>
+      <c r="E18" t="n">
+        <v>210.45</v>
+      </c>
+      <c r="F18" t="n">
+        <v>234.05</v>
+      </c>
+      <c r="G18" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="H18" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I18" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:26:21</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>221.45</v>
+      </c>
+      <c r="D19" t="n">
+        <v>225.74</v>
+      </c>
+      <c r="E19" t="n">
+        <v>202.98</v>
+      </c>
+      <c r="F19" t="n">
+        <v>225.74</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="H19" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I19" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cleaned up and removed redundant code
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2560,6 +2560,120 @@
         <v>83.3</v>
       </c>
       <c r="J55" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>633.66</v>
+      </c>
+      <c r="D56" t="n">
+        <v>666.03</v>
+      </c>
+      <c r="E56" t="n">
+        <v>633.66</v>
+      </c>
+      <c r="F56" t="n">
+        <v>666.03</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="H56" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I56" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="D57" t="n">
+        <v>654.77</v>
+      </c>
+      <c r="E57" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="F57" t="n">
+        <v>646.79</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="H57" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I57" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>623.8</v>
+      </c>
+      <c r="D58" t="n">
+        <v>643.13</v>
+      </c>
+      <c r="E58" t="n">
+        <v>623.8</v>
+      </c>
+      <c r="F58" t="n">
+        <v>632.5700000000001</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H58" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I58" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -2576,7 +2690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4708,6 +4822,120 @@
         <v>83.3</v>
       </c>
       <c r="J55" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>256.8</v>
+      </c>
+      <c r="D56" t="n">
+        <v>275.47</v>
+      </c>
+      <c r="E56" t="n">
+        <v>240.41</v>
+      </c>
+      <c r="F56" t="n">
+        <v>268.89</v>
+      </c>
+      <c r="G56" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="H56" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I56" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>254.91</v>
+      </c>
+      <c r="D57" t="n">
+        <v>267.92</v>
+      </c>
+      <c r="E57" t="n">
+        <v>240.41</v>
+      </c>
+      <c r="F57" t="n">
+        <v>261.53</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="H57" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I57" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>253.02</v>
+      </c>
+      <c r="D58" t="n">
+        <v>267.92</v>
+      </c>
+      <c r="E58" t="n">
+        <v>235.4</v>
+      </c>
+      <c r="F58" t="n">
+        <v>256.08</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="H58" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I58" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -4724,7 +4952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6858,6 +7086,120 @@
       <c r="J55" t="inlineStr">
         <is>
           <t>SELL</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>345.49</v>
+      </c>
+      <c r="D56" t="n">
+        <v>426.92</v>
+      </c>
+      <c r="E56" t="n">
+        <v>345.49</v>
+      </c>
+      <c r="F56" t="n">
+        <v>351.31</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-5.78</v>
+      </c>
+      <c r="H56" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I56" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>342.38</v>
+      </c>
+      <c r="D57" t="n">
+        <v>412.67</v>
+      </c>
+      <c r="E57" t="n">
+        <v>339.59</v>
+      </c>
+      <c r="F57" t="n">
+        <v>339.59</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-8.93</v>
+      </c>
+      <c r="H57" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I57" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>339.26</v>
+      </c>
+      <c r="D58" t="n">
+        <v>412.67</v>
+      </c>
+      <c r="E58" t="n">
+        <v>330.93</v>
+      </c>
+      <c r="F58" t="n">
+        <v>330.93</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-11.25</v>
+      </c>
+      <c r="H58" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I58" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -6872,7 +7214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7881,6 +8223,138 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>226.28</v>
+      </c>
+      <c r="D23" t="n">
+        <v>245.54</v>
+      </c>
+      <c r="E23" t="n">
+        <v>210.67</v>
+      </c>
+      <c r="F23" t="n">
+        <v>245.54</v>
+      </c>
+      <c r="G23" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="H23" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I23" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:31</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>223.46</v>
+      </c>
+      <c r="D24" t="n">
+        <v>234.3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>210.67</v>
+      </c>
+      <c r="F24" t="n">
+        <v>234.3</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="H24" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I24" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-07 19:37:31</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>220.63</v>
+      </c>
+      <c r="D25" t="n">
+        <v>225.98</v>
+      </c>
+      <c r="E25" t="n">
+        <v>203.19</v>
+      </c>
+      <c r="F25" t="n">
+        <v>225.98</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H25" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I25" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refined the data displayed
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2674,6 +2674,120 @@
         <v>83.3</v>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>633.35</v>
+      </c>
+      <c r="D59" t="n">
+        <v>665.51</v>
+      </c>
+      <c r="E59" t="n">
+        <v>633.35</v>
+      </c>
+      <c r="F59" t="n">
+        <v>665.51</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I59" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>628.42</v>
+      </c>
+      <c r="D60" t="n">
+        <v>654.92</v>
+      </c>
+      <c r="E60" t="n">
+        <v>628.42</v>
+      </c>
+      <c r="F60" t="n">
+        <v>646.28</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-1.92</v>
+      </c>
+      <c r="H60" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I60" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>623.5</v>
+      </c>
+      <c r="D61" t="n">
+        <v>643.21</v>
+      </c>
+      <c r="E61" t="n">
+        <v>623.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>632.0700000000001</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-4.08</v>
+      </c>
+      <c r="H61" t="n">
+        <v>658.9299999999999</v>
+      </c>
+      <c r="I61" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -2690,7 +2804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4936,6 +5050,120 @@
         <v>83.3</v>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>256.96</v>
+      </c>
+      <c r="D59" t="n">
+        <v>275.21</v>
+      </c>
+      <c r="E59" t="n">
+        <v>240.24</v>
+      </c>
+      <c r="F59" t="n">
+        <v>269.71</v>
+      </c>
+      <c r="G59" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="H59" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I59" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>255.06</v>
+      </c>
+      <c r="D60" t="n">
+        <v>267.67</v>
+      </c>
+      <c r="E60" t="n">
+        <v>240.24</v>
+      </c>
+      <c r="F60" t="n">
+        <v>262.33</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H60" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I60" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>253.17</v>
+      </c>
+      <c r="D61" t="n">
+        <v>267.67</v>
+      </c>
+      <c r="E61" t="n">
+        <v>235.24</v>
+      </c>
+      <c r="F61" t="n">
+        <v>256.87</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="H61" t="n">
+        <v>258.86</v>
+      </c>
+      <c r="I61" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -4952,7 +5180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7198,6 +7426,120 @@
         <v>81.7</v>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>343.57</v>
+      </c>
+      <c r="D59" t="n">
+        <v>426.48</v>
+      </c>
+      <c r="E59" t="n">
+        <v>343.57</v>
+      </c>
+      <c r="F59" t="n">
+        <v>350.04</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-6.13</v>
+      </c>
+      <c r="H59" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I59" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>340.47</v>
+      </c>
+      <c r="D60" t="n">
+        <v>412.25</v>
+      </c>
+      <c r="E60" t="n">
+        <v>338.36</v>
+      </c>
+      <c r="F60" t="n">
+        <v>338.36</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-9.26</v>
+      </c>
+      <c r="H60" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I60" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:11</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>337.38</v>
+      </c>
+      <c r="D61" t="n">
+        <v>412.25</v>
+      </c>
+      <c r="E61" t="n">
+        <v>329.73</v>
+      </c>
+      <c r="F61" t="n">
+        <v>329.73</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-11.57</v>
+      </c>
+      <c r="H61" t="n">
+        <v>372.88</v>
+      </c>
+      <c r="I61" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -7214,7 +7556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8355,6 +8697,138 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:12</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>225.8</v>
+      </c>
+      <c r="D26" t="n">
+        <v>245.88</v>
+      </c>
+      <c r="E26" t="n">
+        <v>210.89</v>
+      </c>
+      <c r="F26" t="n">
+        <v>245.88</v>
+      </c>
+      <c r="G26" t="n">
+        <v>15.55</v>
+      </c>
+      <c r="H26" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I26" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:12</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>222.98</v>
+      </c>
+      <c r="D27" t="n">
+        <v>234.62</v>
+      </c>
+      <c r="E27" t="n">
+        <v>210.89</v>
+      </c>
+      <c r="F27" t="n">
+        <v>234.62</v>
+      </c>
+      <c r="G27" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="H27" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I27" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-07 20:17:12</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>220.16</v>
+      </c>
+      <c r="D28" t="n">
+        <v>226.29</v>
+      </c>
+      <c r="E28" t="n">
+        <v>203.4</v>
+      </c>
+      <c r="F28" t="n">
+        <v>226.29</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="H28" t="n">
+        <v>212.79</v>
+      </c>
+      <c r="I28" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
better UI/UX for graph
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3157,6 +3157,234 @@
         <v>83.3</v>
       </c>
       <c r="J70" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>638.91</v>
+      </c>
+      <c r="D71" t="n">
+        <v>661.97</v>
+      </c>
+      <c r="E71" t="n">
+        <v>638.91</v>
+      </c>
+      <c r="F71" t="n">
+        <v>658.66</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="H71" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I71" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>633.8200000000001</v>
+      </c>
+      <c r="D72" t="n">
+        <v>642.42</v>
+      </c>
+      <c r="E72" t="n">
+        <v>633.8200000000001</v>
+      </c>
+      <c r="F72" t="n">
+        <v>639.21</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-3.04</v>
+      </c>
+      <c r="H72" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I72" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>628.74</v>
+      </c>
+      <c r="D73" t="n">
+        <v>642.42</v>
+      </c>
+      <c r="E73" t="n">
+        <v>624.83</v>
+      </c>
+      <c r="F73" t="n">
+        <v>624.83</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-5.22</v>
+      </c>
+      <c r="H73" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I73" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>638.8200000000001</v>
+      </c>
+      <c r="D74" t="n">
+        <v>662.84</v>
+      </c>
+      <c r="E74" t="n">
+        <v>638.8200000000001</v>
+      </c>
+      <c r="F74" t="n">
+        <v>659.35</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H74" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I74" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>633.74</v>
+      </c>
+      <c r="D75" t="n">
+        <v>643.26</v>
+      </c>
+      <c r="E75" t="n">
+        <v>633.74</v>
+      </c>
+      <c r="F75" t="n">
+        <v>639.88</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-2.93</v>
+      </c>
+      <c r="H75" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I75" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>628.66</v>
+      </c>
+      <c r="D76" t="n">
+        <v>643.26</v>
+      </c>
+      <c r="E76" t="n">
+        <v>625.11</v>
+      </c>
+      <c r="F76" t="n">
+        <v>625.49</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-5.12</v>
+      </c>
+      <c r="H76" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I76" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J76" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -3173,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5845,6 +6073,234 @@
         <v>81.7</v>
       </c>
       <c r="J70" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>265.66</v>
+      </c>
+      <c r="D71" t="n">
+        <v>272.85</v>
+      </c>
+      <c r="E71" t="n">
+        <v>244.62</v>
+      </c>
+      <c r="F71" t="n">
+        <v>265.72</v>
+      </c>
+      <c r="G71" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="H71" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I71" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>263.46</v>
+      </c>
+      <c r="D72" t="n">
+        <v>264.44</v>
+      </c>
+      <c r="E72" t="n">
+        <v>244.62</v>
+      </c>
+      <c r="F72" t="n">
+        <v>257.52</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="H72" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I72" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:04</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>261.25</v>
+      </c>
+      <c r="D73" t="n">
+        <v>264.44</v>
+      </c>
+      <c r="E73" t="n">
+        <v>238.87</v>
+      </c>
+      <c r="F73" t="n">
+        <v>251.47</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="H73" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I73" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>265.73</v>
+      </c>
+      <c r="D74" t="n">
+        <v>272.4</v>
+      </c>
+      <c r="E74" t="n">
+        <v>244.13</v>
+      </c>
+      <c r="F74" t="n">
+        <v>265.72</v>
+      </c>
+      <c r="G74" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="H74" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I74" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>263.52</v>
+      </c>
+      <c r="D75" t="n">
+        <v>264</v>
+      </c>
+      <c r="E75" t="n">
+        <v>244.13</v>
+      </c>
+      <c r="F75" t="n">
+        <v>257.52</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="H75" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I75" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>261.31</v>
+      </c>
+      <c r="D76" t="n">
+        <v>264</v>
+      </c>
+      <c r="E76" t="n">
+        <v>238.38</v>
+      </c>
+      <c r="F76" t="n">
+        <v>251.47</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="H76" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I76" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J76" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -5861,7 +6317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8535,6 +8991,234 @@
       <c r="J70" t="inlineStr">
         <is>
           <t>HOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>339.63</v>
+      </c>
+      <c r="D71" t="n">
+        <v>444.89</v>
+      </c>
+      <c r="E71" t="n">
+        <v>339.63</v>
+      </c>
+      <c r="F71" t="n">
+        <v>392.59</v>
+      </c>
+      <c r="G71" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="H71" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I71" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>336.55</v>
+      </c>
+      <c r="D72" t="n">
+        <v>429.97</v>
+      </c>
+      <c r="E72" t="n">
+        <v>336.55</v>
+      </c>
+      <c r="F72" t="n">
+        <v>379.42</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="H72" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I72" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>333.47</v>
+      </c>
+      <c r="D73" t="n">
+        <v>429.97</v>
+      </c>
+      <c r="E73" t="n">
+        <v>333.47</v>
+      </c>
+      <c r="F73" t="n">
+        <v>369.69</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="H73" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I73" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>339.06</v>
+      </c>
+      <c r="D74" t="n">
+        <v>441.29</v>
+      </c>
+      <c r="E74" t="n">
+        <v>339.06</v>
+      </c>
+      <c r="F74" t="n">
+        <v>393.78</v>
+      </c>
+      <c r="G74" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="H74" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I74" t="n">
+        <v>85</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>335.99</v>
+      </c>
+      <c r="D75" t="n">
+        <v>426.48</v>
+      </c>
+      <c r="E75" t="n">
+        <v>335.99</v>
+      </c>
+      <c r="F75" t="n">
+        <v>380.57</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="H75" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I75" t="n">
+        <v>85</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:18</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>332.91</v>
+      </c>
+      <c r="D76" t="n">
+        <v>426.48</v>
+      </c>
+      <c r="E76" t="n">
+        <v>332.91</v>
+      </c>
+      <c r="F76" t="n">
+        <v>370.81</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="H76" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I76" t="n">
+        <v>85</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
         </is>
       </c>
     </row>
@@ -8549,7 +9233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9967,6 +10651,234 @@
         <v>85</v>
       </c>
       <c r="J37" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>220.51</v>
+      </c>
+      <c r="D38" t="n">
+        <v>236.57</v>
+      </c>
+      <c r="E38" t="n">
+        <v>215.8</v>
+      </c>
+      <c r="F38" t="n">
+        <v>236.57</v>
+      </c>
+      <c r="G38" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H38" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I38" t="n">
+        <v>85</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>217.95</v>
+      </c>
+      <c r="D39" t="n">
+        <v>226.46</v>
+      </c>
+      <c r="E39" t="n">
+        <v>215.8</v>
+      </c>
+      <c r="F39" t="n">
+        <v>226.46</v>
+      </c>
+      <c r="G39" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="H39" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I39" t="n">
+        <v>85</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>215.39</v>
+      </c>
+      <c r="D40" t="n">
+        <v>220.62</v>
+      </c>
+      <c r="E40" t="n">
+        <v>208.68</v>
+      </c>
+      <c r="F40" t="n">
+        <v>218.99</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H40" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I40" t="n">
+        <v>85</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>220.49</v>
+      </c>
+      <c r="D41" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="E41" t="n">
+        <v>215.97</v>
+      </c>
+      <c r="F41" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="G41" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="H41" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I41" t="n">
+        <v>85</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>217.93</v>
+      </c>
+      <c r="D42" t="n">
+        <v>226.36</v>
+      </c>
+      <c r="E42" t="n">
+        <v>215.97</v>
+      </c>
+      <c r="F42" t="n">
+        <v>226.36</v>
+      </c>
+      <c r="G42" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="H42" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I42" t="n">
+        <v>85</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>215.37</v>
+      </c>
+      <c r="D43" t="n">
+        <v>220.77</v>
+      </c>
+      <c r="E43" t="n">
+        <v>208.85</v>
+      </c>
+      <c r="F43" t="n">
+        <v>218.89</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H43" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I43" t="n">
+        <v>85</v>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -9983,7 +10895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10380,6 +11292,234 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>610.62</v>
+      </c>
+      <c r="D11" t="n">
+        <v>689.89</v>
+      </c>
+      <c r="E11" t="n">
+        <v>590.33</v>
+      </c>
+      <c r="F11" t="n">
+        <v>689.89</v>
+      </c>
+      <c r="G11" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="H11" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I11" t="n">
+        <v>80</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>597.95</v>
+      </c>
+      <c r="D12" t="n">
+        <v>638.55</v>
+      </c>
+      <c r="E12" t="n">
+        <v>590.33</v>
+      </c>
+      <c r="F12" t="n">
+        <v>638.55</v>
+      </c>
+      <c r="G12" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="H12" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I12" t="n">
+        <v>80</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-08 16:52:05</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>585.28</v>
+      </c>
+      <c r="D13" t="n">
+        <v>638.54</v>
+      </c>
+      <c r="E13" t="n">
+        <v>555.25</v>
+      </c>
+      <c r="F13" t="n">
+        <v>600.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="H13" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I13" t="n">
+        <v>80</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>611.11</v>
+      </c>
+      <c r="D14" t="n">
+        <v>689.1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>589.63</v>
+      </c>
+      <c r="F14" t="n">
+        <v>689.1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>19.83</v>
+      </c>
+      <c r="H14" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I14" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>598.4299999999999</v>
+      </c>
+      <c r="D15" t="n">
+        <v>637.8200000000001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>589.63</v>
+      </c>
+      <c r="F15" t="n">
+        <v>637.8200000000001</v>
+      </c>
+      <c r="G15" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="H15" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I15" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-08 17:09:19</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>585.76</v>
+      </c>
+      <c r="D16" t="n">
+        <v>636.25</v>
+      </c>
+      <c r="E16" t="n">
+        <v>554.59</v>
+      </c>
+      <c r="F16" t="n">
+        <v>599.92</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="H16" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I16" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ran this for 1 hour to limit test
</commit_message>
<xml_diff>
--- a/stock_predictions.xlsx
+++ b/stock_predictions.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3385,6 +3385,120 @@
         <v>83.3</v>
       </c>
       <c r="J76" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>638.8200000000001</v>
+      </c>
+      <c r="D77" t="n">
+        <v>663.02</v>
+      </c>
+      <c r="E77" t="n">
+        <v>638.8200000000001</v>
+      </c>
+      <c r="F77" t="n">
+        <v>659.4</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H77" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I77" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>633.74</v>
+      </c>
+      <c r="D78" t="n">
+        <v>643.4400000000001</v>
+      </c>
+      <c r="E78" t="n">
+        <v>633.74</v>
+      </c>
+      <c r="F78" t="n">
+        <v>639.9299999999999</v>
+      </c>
+      <c r="G78" t="n">
+        <v>-2.93</v>
+      </c>
+      <c r="H78" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I78" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>628.66</v>
+      </c>
+      <c r="D79" t="n">
+        <v>643.4400000000001</v>
+      </c>
+      <c r="E79" t="n">
+        <v>625.02</v>
+      </c>
+      <c r="F79" t="n">
+        <v>625.54</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="H79" t="n">
+        <v>659.22</v>
+      </c>
+      <c r="I79" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J79" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
@@ -3401,7 +3515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6301,6 +6415,120 @@
         <v>83.3</v>
       </c>
       <c r="J76" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>265.89</v>
+      </c>
+      <c r="D77" t="n">
+        <v>272.25</v>
+      </c>
+      <c r="E77" t="n">
+        <v>243.83</v>
+      </c>
+      <c r="F77" t="n">
+        <v>265.59</v>
+      </c>
+      <c r="G77" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="H77" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I77" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>263.68</v>
+      </c>
+      <c r="D78" t="n">
+        <v>263.86</v>
+      </c>
+      <c r="E78" t="n">
+        <v>243.83</v>
+      </c>
+      <c r="F78" t="n">
+        <v>257.4</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="H78" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I78" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>261.47</v>
+      </c>
+      <c r="D79" t="n">
+        <v>263.86</v>
+      </c>
+      <c r="E79" t="n">
+        <v>238.1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>251.35</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="H79" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I79" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J79" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -6317,7 +6545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9217,6 +9445,120 @@
         <v>85</v>
       </c>
       <c r="J76" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>338.32</v>
+      </c>
+      <c r="D77" t="n">
+        <v>440.41</v>
+      </c>
+      <c r="E77" t="n">
+        <v>338.32</v>
+      </c>
+      <c r="F77" t="n">
+        <v>394.18</v>
+      </c>
+      <c r="G77" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="H77" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I77" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>335.25</v>
+      </c>
+      <c r="D78" t="n">
+        <v>425.63</v>
+      </c>
+      <c r="E78" t="n">
+        <v>335.25</v>
+      </c>
+      <c r="F78" t="n">
+        <v>380.96</v>
+      </c>
+      <c r="G78" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="H78" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I78" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:03</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>332.19</v>
+      </c>
+      <c r="D79" t="n">
+        <v>425.63</v>
+      </c>
+      <c r="E79" t="n">
+        <v>332.19</v>
+      </c>
+      <c r="F79" t="n">
+        <v>371.19</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="H79" t="n">
+        <v>372.29</v>
+      </c>
+      <c r="I79" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J79" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -9233,7 +9575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10879,6 +11221,120 @@
         <v>85</v>
       </c>
       <c r="J43" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>220.52</v>
+      </c>
+      <c r="D44" t="n">
+        <v>236.42</v>
+      </c>
+      <c r="E44" t="n">
+        <v>215.98</v>
+      </c>
+      <c r="F44" t="n">
+        <v>236.42</v>
+      </c>
+      <c r="G44" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H44" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I44" t="n">
+        <v>85</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>217.96</v>
+      </c>
+      <c r="D45" t="n">
+        <v>226.32</v>
+      </c>
+      <c r="E45" t="n">
+        <v>215.98</v>
+      </c>
+      <c r="F45" t="n">
+        <v>226.32</v>
+      </c>
+      <c r="G45" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="H45" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I45" t="n">
+        <v>85</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>215.39</v>
+      </c>
+      <c r="D46" t="n">
+        <v>220.93</v>
+      </c>
+      <c r="E46" t="n">
+        <v>208.86</v>
+      </c>
+      <c r="F46" t="n">
+        <v>218.85</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="H46" t="n">
+        <v>213.77</v>
+      </c>
+      <c r="I46" t="n">
+        <v>85</v>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
         </is>
@@ -10895,7 +11351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11520,6 +11976,120 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Best Case</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>611.08</v>
+      </c>
+      <c r="D17" t="n">
+        <v>688.99</v>
+      </c>
+      <c r="E17" t="n">
+        <v>589.63</v>
+      </c>
+      <c r="F17" t="n">
+        <v>688.99</v>
+      </c>
+      <c r="G17" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="H17" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I17" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Average Case</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>598.4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>637.72</v>
+      </c>
+      <c r="E18" t="n">
+        <v>589.63</v>
+      </c>
+      <c r="F18" t="n">
+        <v>637.72</v>
+      </c>
+      <c r="G18" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H18" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I18" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-08 22:12:04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Worst Case</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>585.72</v>
+      </c>
+      <c r="D19" t="n">
+        <v>635.85</v>
+      </c>
+      <c r="E19" t="n">
+        <v>554.59</v>
+      </c>
+      <c r="F19" t="n">
+        <v>599.8200000000001</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="H19" t="n">
+        <v>575.05</v>
+      </c>
+      <c r="I19" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>